<commit_message>
Fix clipped names in assembly exports
</commit_message>
<xml_diff>
--- a/exact-templates/default-assembly.xlsx
+++ b/exact-templates/default-assembly.xlsx
@@ -1106,13 +1106,13 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.5" style="3" customWidth="1"/>
-    <col min="2" max="2" width="12" style="3" customWidth="1"/>
-    <col min="3" max="3" width="14" style="3" customWidth="1"/>
+    <col min="2" max="2" width="18" style="3" customWidth="1"/>
+    <col min="3" max="3" width="16" style="3" customWidth="1"/>
     <col min="4" max="4" width="18" style="3" customWidth="1"/>
     <col min="5" max="5" width="6.5" style="3" customWidth="1"/>
     <col min="6" max="6" width="6.5" style="4" customWidth="1"/>
     <col min="7" max="7" width="8" style="3" customWidth="1"/>
-    <col min="8" max="8" width="7" style="3" customWidth="1"/>
+    <col min="8" max="8" width="8" style="3" customWidth="1"/>
     <col min="9" max="9" width="12" style="3" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>